<commit_message>
Update AA versus NSA Functions.xlsx
Changed Speed support.
</commit_message>
<xml_diff>
--- a/New-Scale-Analytics-Rules/AA versus NSA Functions.xlsx
+++ b/New-Scale-Analytics-Rules/AA versus NSA Functions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yyexabeam-my.sharepoint.com/personal/vaughn_adams_exabeam_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yyexabeam-my.sharepoint.com/personal/vaughn_adams_exabeam_com/Documents/Documents/GitHub/new-scale-content-hub/New-Scale-Analytics-Rules/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{89E288A3-9A8D-4C35-A918-5DCDC7728055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{89E288A3-9A8D-4C35-A918-5DCDC7728055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D62827EB-183E-4CDF-BC51-57C685317DD8}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{8164C3EA-DD38-490E-B173-6AA108847BAB}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{8164C3EA-DD38-490E-B173-6AA108847BAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -853,6 +853,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FC101D1-202B-4B77-8CA2-312DDDAA5E47}">
   <dimension ref="A1:D1006"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="30.5546875" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="16.109375" customWidth="1"/>
+    <col min="4" max="4" width="44.5546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="58.2" thickBot="1">
       <c r="A1" s="1" t="s">
@@ -1876,7 +1882,7 @@
         <v>1</v>
       </c>
       <c r="C86" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D86" s="2"/>
     </row>

</xml_diff>